<commit_message>
🐛 fix: fixed xansha excels templates
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/XANSHA/HOTEL/Tax Invoice.xlsx
+++ b/apps/excel-service/templates/XANSHA/HOTEL/Tax Invoice.xlsx
@@ -97,7 +97,7 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">БИН и адрес места нахождения получателя:</t>
+      <t xml:space="preserve">БИН и адрес места нахождения грузополучателя:</t>
     </r>
     <r>
       <rPr>
@@ -116,7 +116,7 @@
         <color theme="1"/>
         <rFont val="Arial"/>
       </rPr>
-      <t xml:space="preserve">БИН и адрес места нахождения получателя: </t>
+      <t xml:space="preserve">БИН и Банк грузополучателя: </t>
     </r>
     <r>
       <rPr>

</xml_diff>